<commit_message>
n8n board refresh 2026-10-15T17:42:48Z
</commit_message>
<xml_diff>
--- a/app/reports/BBD_research.xlsx
+++ b/app/reports/BBD_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-27 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-15 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>3.41</v>
+        <v>4.06</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.05184000015258789</v>
+        <v>0.05085000038146972</v>
       </c>
     </row>
     <row r="6">
@@ -1208,7 +1208,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>10589177393.54839</v>
+        <v>11175563728.07882</v>
       </c>
     </row>
     <row r="36">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>3.41</v>
+        <v>4.06</v>
       </c>
     </row>
     <row r="38">
@@ -1508,14 +1508,14 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>36109094912</v>
+        <v>45372788736</v>
       </c>
       <c r="D5" s="31" t="n">
-        <v>8.119999999999999</v>
+        <v>13.53</v>
       </c>
       <c r="E5" s="31" t="n"/>
       <c r="F5" s="31" t="n">
-        <v>6.39</v>
+        <v>6.47</v>
       </c>
     </row>
     <row r="6">
@@ -1530,10 +1530,10 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>2685712384</v>
+        <v>2595848192</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v>11.954545</v>
+        <v>9.9296875</v>
       </c>
       <c r="E6" s="33" t="n"/>
       <c r="F6" s="33" t="n">
@@ -1543,44 +1543,44 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BBDO</t>
+          <t>BCH</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Banco Bradesco Sa</t>
+          <t>Banco De Chile</t>
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>32826447872</v>
+        <v>19723585536</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>7.3809524</v>
+        <v>15.019231</v>
       </c>
       <c r="E7" s="33" t="n"/>
-      <c r="F7" s="33" t="n">
-        <v>6.353</v>
-      </c>
+      <c r="F7" s="33" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BCH</t>
+          <t>BDORY</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Banco De Chile</t>
+          <t>Banco Do Brasil SA</t>
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>21233790976</v>
+        <v>27459917824</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>17.020243</v>
+        <v>12.333334</v>
       </c>
       <c r="E8" s="33" t="n"/>
-      <c r="F8" s="33" t="n"/>
+      <c r="F8" s="33" t="n">
+        <v>10.826</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1594,14 +1594,14 @@
         </is>
       </c>
       <c r="C9" s="32" t="n">
-        <v>4402841600</v>
+        <v>4122789120</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>17.477158</v>
+        <v>13.603377</v>
       </c>
       <c r="E9" s="33" t="n"/>
       <c r="F9" s="33" t="n">
-        <v>-0.435</v>
+        <v>-0.386</v>
       </c>
     </row>
     <row r="10">
@@ -1616,10 +1616,10 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>16192233472</v>
+        <v>15351292928</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>13.971544</v>
+        <v>12.581081</v>
       </c>
       <c r="E10" s="33" t="n"/>
       <c r="F10" s="33" t="n"/>
@@ -1636,58 +1636,58 @@
         </is>
       </c>
       <c r="C11" s="32" t="n">
-        <v>43128160256</v>
+        <v>20909381632</v>
       </c>
       <c r="D11" s="33" t="n">
-        <v>16.941177</v>
+        <v>16.924242</v>
       </c>
       <c r="E11" s="33" t="n"/>
       <c r="F11" s="33" t="n">
-        <v>3.519</v>
+        <v>3.512</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>GGAL</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Deutsche Bank AG</t>
+          <t>Grupo Financiero Galicia S.A.</t>
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>68715032576</v>
+        <v>6079989760</v>
       </c>
       <c r="D12" s="33" t="n">
-        <v>9.778074999999999</v>
+        <v>41.720932</v>
       </c>
       <c r="E12" s="33" t="n"/>
       <c r="F12" s="33" t="n">
-        <v>-0.698</v>
+        <v>0.057</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GGAL</t>
+          <t>ITAUCL.SN</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Grupo Financiero Galicia S.A.</t>
+          <t>BANCO ITAU CHILE</t>
         </is>
       </c>
       <c r="C13" s="32" t="n">
-        <v>6564626432</v>
+        <v>5040739713024</v>
       </c>
       <c r="D13" s="33" t="n">
-        <v>110.68572</v>
+        <v>12.540366</v>
       </c>
       <c r="E13" s="33" t="n"/>
       <c r="F13" s="33" t="n">
-        <v>0.058</v>
+        <v>11.391</v>
       </c>
     </row>
     <row r="15">
@@ -1735,11 +1735,11 @@
         </is>
       </c>
       <c r="D17" s="35" t="n">
-        <v>0.167</v>
+        <v>0.5</v>
       </c>
       <c r="E17" s="35" t="n"/>
       <c r="F17" s="35" t="n">
-        <v>1</v>
+        <v>0.667</v>
       </c>
     </row>
     <row r="18">

</xml_diff>